<commit_message>
Updated w/ Non Cumulative & More Previous Years
Info from Sales Analysis Meeting.xlsx
</commit_message>
<xml_diff>
--- a/Notebooks/sales_analysis_data.xlsx
+++ b/Notebooks/sales_analysis_data.xlsx
@@ -5,18 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HHrbek\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\MACOLA\macapps\REPORTS\PURCHASING-XIV\Personal\Code\Notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FAF72BCB-19BD-4153-B7F3-B9EA9778F748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3F6DE0-D0F1-4F3E-BC1A-63EE7D52226F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{8B61463E-2888-4AE7-B526-3393957A0401}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{8B61463E-2888-4AE7-B526-3393957A0401}"/>
   </bookViews>
   <sheets>
     <sheet name="2023" sheetId="1" r:id="rId1"/>
     <sheet name="2024" sheetId="2" r:id="rId2"/>
     <sheet name="2025" sheetId="3" r:id="rId3"/>
     <sheet name="2026" sheetId="4" r:id="rId4"/>
+    <sheet name="noncumulative" sheetId="5" r:id="rId5"/>
+    <sheet name="other_years" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="20">
   <si>
     <t>2023</t>
   </si>
@@ -1140,4 +1142,941 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA8CF6F5-D031-4840-A14D-E801A891D7F1}">
+  <dimension ref="A1:N19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>852827.79</v>
+      </c>
+      <c r="C2">
+        <v>1941736.86</v>
+      </c>
+      <c r="D2">
+        <v>2877487.69</v>
+      </c>
+      <c r="E2">
+        <v>3609987.3</v>
+      </c>
+      <c r="F2">
+        <v>4825078.24</v>
+      </c>
+      <c r="G2">
+        <v>5866636.1299999999</v>
+      </c>
+      <c r="H2">
+        <v>6423941.4299999997</v>
+      </c>
+      <c r="I2">
+        <v>7540840.1399999997</v>
+      </c>
+      <c r="J2">
+        <v>8338579.6799999997</v>
+      </c>
+      <c r="K2">
+        <v>9319105.4800000004</v>
+      </c>
+      <c r="L2">
+        <v>10067554.609999999</v>
+      </c>
+      <c r="M2">
+        <v>10792586.67</v>
+      </c>
+      <c r="N2">
+        <v>10792586.67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>806590.68</v>
+      </c>
+      <c r="C3">
+        <v>1625399.05</v>
+      </c>
+      <c r="D3">
+        <v>2612447.2000000002</v>
+      </c>
+      <c r="E3">
+        <v>3706819.85</v>
+      </c>
+      <c r="F3">
+        <v>4686154.96</v>
+      </c>
+      <c r="G3">
+        <v>5659758.9400000004</v>
+      </c>
+      <c r="H3">
+        <v>6477805.1399999997</v>
+      </c>
+      <c r="I3">
+        <v>7489595.9800000004</v>
+      </c>
+      <c r="J3">
+        <v>8386523.3899999997</v>
+      </c>
+      <c r="K3">
+        <v>9365238.1999999993</v>
+      </c>
+      <c r="L3">
+        <v>10223218.640000001</v>
+      </c>
+      <c r="M3">
+        <v>11074512.939999999</v>
+      </c>
+      <c r="N3">
+        <v>11074512.939999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4">
+        <v>750000</v>
+      </c>
+      <c r="C4">
+        <v>1550000</v>
+      </c>
+      <c r="D4">
+        <v>2740000</v>
+      </c>
+      <c r="E4">
+        <v>3930000</v>
+      </c>
+      <c r="F4">
+        <v>5120000</v>
+      </c>
+      <c r="G4">
+        <v>5920000</v>
+      </c>
+      <c r="H4">
+        <v>7110000</v>
+      </c>
+      <c r="I4">
+        <v>8300000</v>
+      </c>
+      <c r="J4">
+        <v>9490000</v>
+      </c>
+      <c r="K4">
+        <v>10680000</v>
+      </c>
+      <c r="L4">
+        <v>11870000</v>
+      </c>
+      <c r="M4">
+        <v>12620000</v>
+      </c>
+      <c r="N4">
+        <v>12620000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>6</v>
+      </c>
+      <c r="H6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" t="s">
+        <v>9</v>
+      </c>
+      <c r="K6" t="s">
+        <v>10</v>
+      </c>
+      <c r="L6" t="s">
+        <v>11</v>
+      </c>
+      <c r="M6" t="s">
+        <v>12</v>
+      </c>
+      <c r="N6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>844942.9600000002</v>
+      </c>
+      <c r="C7">
+        <v>992578.01</v>
+      </c>
+      <c r="D7">
+        <v>755367.04</v>
+      </c>
+      <c r="E7">
+        <v>1069724.7099999997</v>
+      </c>
+      <c r="F7">
+        <v>891714.06999999983</v>
+      </c>
+      <c r="G7">
+        <v>1147584.94</v>
+      </c>
+      <c r="H7">
+        <v>1015956.7099999998</v>
+      </c>
+      <c r="I7">
+        <v>1033703.9100000003</v>
+      </c>
+      <c r="J7">
+        <v>960939.77</v>
+      </c>
+      <c r="K7">
+        <v>1139232.28</v>
+      </c>
+      <c r="L7">
+        <v>1387232.7599999995</v>
+      </c>
+      <c r="M7">
+        <v>1218408.8299999998</v>
+      </c>
+      <c r="N7">
+        <v>12457385.99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>881453.75999999989</v>
+      </c>
+      <c r="C8">
+        <v>734697.66</v>
+      </c>
+      <c r="D8">
+        <v>780683.81</v>
+      </c>
+      <c r="E8">
+        <v>942485.29</v>
+      </c>
+      <c r="F8">
+        <v>924715.83000000007</v>
+      </c>
+      <c r="G8">
+        <v>1054174.9100000001</v>
+      </c>
+      <c r="H8">
+        <v>1023904.2600000001</v>
+      </c>
+      <c r="I8">
+        <v>1010126.41</v>
+      </c>
+      <c r="J8">
+        <v>1063610.6299999999</v>
+      </c>
+      <c r="K8">
+        <v>1024897.2599999999</v>
+      </c>
+      <c r="L8">
+        <v>1099864.56</v>
+      </c>
+      <c r="M8">
+        <v>1014224.02</v>
+      </c>
+      <c r="N8">
+        <v>11554838.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>900000</v>
+      </c>
+      <c r="C9">
+        <v>900000</v>
+      </c>
+      <c r="D9">
+        <v>1021450</v>
+      </c>
+      <c r="E9">
+        <v>1035000</v>
+      </c>
+      <c r="F9">
+        <v>1035000</v>
+      </c>
+      <c r="G9">
+        <v>1075000</v>
+      </c>
+      <c r="H9">
+        <v>966254.92424242466</v>
+      </c>
+      <c r="I9">
+        <v>1061924.9999999967</v>
+      </c>
+      <c r="J9">
+        <v>1069595.0757575766</v>
+      </c>
+      <c r="K9">
+        <v>966254.92424242664</v>
+      </c>
+      <c r="L9">
+        <v>1082595.0757575766</v>
+      </c>
+      <c r="M9">
+        <v>886924.99999999965</v>
+      </c>
+      <c r="N9">
+        <v>12000000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C11" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>5</v>
+      </c>
+      <c r="G11" t="s">
+        <v>6</v>
+      </c>
+      <c r="H11" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" t="s">
+        <v>8</v>
+      </c>
+      <c r="J11" t="s">
+        <v>9</v>
+      </c>
+      <c r="K11" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" t="s">
+        <v>11</v>
+      </c>
+      <c r="M11" t="s">
+        <v>12</v>
+      </c>
+      <c r="N11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>1445682.8499999999</v>
+      </c>
+      <c r="C12">
+        <v>1191876.03</v>
+      </c>
+      <c r="D12">
+        <v>1174588.1499999999</v>
+      </c>
+      <c r="E12">
+        <v>1215708.28</v>
+      </c>
+      <c r="F12">
+        <v>1236752.28</v>
+      </c>
+      <c r="G12">
+        <v>928485.44</v>
+      </c>
+      <c r="H12">
+        <v>1199649.6399999999</v>
+      </c>
+      <c r="I12">
+        <v>1023184.73</v>
+      </c>
+      <c r="J12">
+        <v>1049463.6800000002</v>
+      </c>
+      <c r="K12">
+        <v>1095336.7200000002</v>
+      </c>
+      <c r="L12">
+        <v>1040875.5700000001</v>
+      </c>
+      <c r="M12">
+        <v>849365.89000000025</v>
+      </c>
+      <c r="N12">
+        <v>13450969.26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13">
+        <v>982336.6100000001</v>
+      </c>
+      <c r="C13">
+        <v>1064614.17</v>
+      </c>
+      <c r="D13">
+        <v>987903.93999999983</v>
+      </c>
+      <c r="E13">
+        <v>1197538.8600000001</v>
+      </c>
+      <c r="F13">
+        <v>1202583.6100000001</v>
+      </c>
+      <c r="G13">
+        <v>1263727.48</v>
+      </c>
+      <c r="H13">
+        <v>1152111.8499999999</v>
+      </c>
+      <c r="I13">
+        <v>1238928.7300000002</v>
+      </c>
+      <c r="J13">
+        <v>1201686.42</v>
+      </c>
+      <c r="K13">
+        <v>1217526.8800000004</v>
+      </c>
+      <c r="L13">
+        <v>1175288.8</v>
+      </c>
+      <c r="M13">
+        <v>947728.82</v>
+      </c>
+      <c r="N13">
+        <v>13631976.17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14">
+        <v>920940</v>
+      </c>
+      <c r="C14">
+        <v>945624</v>
+      </c>
+      <c r="D14">
+        <v>967940</v>
+      </c>
+      <c r="E14">
+        <v>1143578</v>
+      </c>
+      <c r="F14">
+        <v>1093578</v>
+      </c>
+      <c r="G14">
+        <v>1093578</v>
+      </c>
+      <c r="H14">
+        <v>1060669</v>
+      </c>
+      <c r="I14">
+        <v>1131035</v>
+      </c>
+      <c r="J14">
+        <v>1131035</v>
+      </c>
+      <c r="K14">
+        <v>1115354</v>
+      </c>
+      <c r="L14">
+        <v>1115354</v>
+      </c>
+      <c r="M14">
+        <v>981314</v>
+      </c>
+      <c r="N14">
+        <v>12699999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" t="s">
+        <v>5</v>
+      </c>
+      <c r="G16" t="s">
+        <v>6</v>
+      </c>
+      <c r="H16" t="s">
+        <v>7</v>
+      </c>
+      <c r="I16" t="s">
+        <v>8</v>
+      </c>
+      <c r="J16" t="s">
+        <v>9</v>
+      </c>
+      <c r="K16" t="s">
+        <v>10</v>
+      </c>
+      <c r="L16" t="s">
+        <v>11</v>
+      </c>
+      <c r="M16" t="s">
+        <v>12</v>
+      </c>
+      <c r="N16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17">
+        <v>955153.66999999981</v>
+      </c>
+      <c r="C17">
+        <v>960511.59</v>
+      </c>
+      <c r="D17">
+        <v>1234337.8099999998</v>
+      </c>
+      <c r="E17">
+        <v>1363198</v>
+      </c>
+      <c r="N17">
+        <v>4513201.07</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>15</v>
+      </c>
+      <c r="B18">
+        <v>985408.35</v>
+      </c>
+      <c r="C18">
+        <v>1008835.0900000002</v>
+      </c>
+      <c r="D18">
+        <v>1134311.55</v>
+      </c>
+      <c r="E18">
+        <v>1280154.81</v>
+      </c>
+      <c r="N18">
+        <v>4408709.8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>16</v>
+      </c>
+      <c r="B19">
+        <v>973389</v>
+      </c>
+      <c r="C19">
+        <v>983442</v>
+      </c>
+      <c r="D19">
+        <v>1146319</v>
+      </c>
+      <c r="E19">
+        <v>1287077</v>
+      </c>
+      <c r="F19">
+        <v>1287077</v>
+      </c>
+      <c r="G19">
+        <v>1277017</v>
+      </c>
+      <c r="H19">
+        <v>1256912</v>
+      </c>
+      <c r="I19">
+        <v>1146319</v>
+      </c>
+      <c r="J19">
+        <v>1226747</v>
+      </c>
+      <c r="K19">
+        <v>1226747</v>
+      </c>
+      <c r="L19">
+        <v>1166026</v>
+      </c>
+      <c r="M19">
+        <v>13981626</v>
+      </c>
+      <c r="N19">
+        <v>13981626</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5764B6C5-DE29-4DCD-9666-E9542FDC04F7}">
+  <dimension ref="A1:N6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2022</v>
+      </c>
+      <c r="B2">
+        <v>1037420.61</v>
+      </c>
+      <c r="C2">
+        <v>1811271.77</v>
+      </c>
+      <c r="D2">
+        <v>2781796.5260000001</v>
+      </c>
+      <c r="E2">
+        <v>3698798.696</v>
+      </c>
+      <c r="F2">
+        <v>5051560.3459999999</v>
+      </c>
+      <c r="G2">
+        <v>5847928.6359999999</v>
+      </c>
+      <c r="H2">
+        <v>6867308.4059999995</v>
+      </c>
+      <c r="I2">
+        <v>7840905.6359999999</v>
+      </c>
+      <c r="J2">
+        <v>8910614.8460000008</v>
+      </c>
+      <c r="K2">
+        <v>9478940.8260000013</v>
+      </c>
+      <c r="L2">
+        <v>10203898.496000001</v>
+      </c>
+      <c r="M2">
+        <v>10969800.626000002</v>
+      </c>
+      <c r="N2">
+        <v>10969800.626000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2021</v>
+      </c>
+      <c r="B3">
+        <v>1247663.42</v>
+      </c>
+      <c r="C3">
+        <v>1903942.39</v>
+      </c>
+      <c r="D3">
+        <v>3036239.2199999997</v>
+      </c>
+      <c r="E3">
+        <v>3813161.3499999996</v>
+      </c>
+      <c r="F3">
+        <v>4518330.38</v>
+      </c>
+      <c r="G3">
+        <v>5245290.5199999996</v>
+      </c>
+      <c r="H3">
+        <v>5987391.0399999991</v>
+      </c>
+      <c r="I3">
+        <v>6843265.3499999996</v>
+      </c>
+      <c r="J3">
+        <v>7739962.7699999996</v>
+      </c>
+      <c r="K3">
+        <v>8475881.9100000001</v>
+      </c>
+      <c r="L3">
+        <v>9198198.6300000008</v>
+      </c>
+      <c r="M3">
+        <v>10189956.700000001</v>
+      </c>
+      <c r="N3">
+        <v>10189956.700000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2020</v>
+      </c>
+      <c r="B4">
+        <v>706328.87</v>
+      </c>
+      <c r="C4">
+        <v>1526726.8</v>
+      </c>
+      <c r="D4">
+        <v>2722010.8200000003</v>
+      </c>
+      <c r="E4">
+        <v>4107415.0900000003</v>
+      </c>
+      <c r="F4">
+        <v>5785756.5</v>
+      </c>
+      <c r="G4">
+        <v>6885169.6699999999</v>
+      </c>
+      <c r="H4">
+        <v>7917466.6799999997</v>
+      </c>
+      <c r="I4">
+        <v>8717838.5199999996</v>
+      </c>
+      <c r="J4">
+        <v>9711868.3899999987</v>
+      </c>
+      <c r="K4">
+        <v>10943113.199999999</v>
+      </c>
+      <c r="L4">
+        <v>11813437.699999999</v>
+      </c>
+      <c r="M4">
+        <v>12373495.699999999</v>
+      </c>
+      <c r="N4">
+        <v>12373495.699999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>2019</v>
+      </c>
+      <c r="B5">
+        <v>1177735.3799999999</v>
+      </c>
+      <c r="C5">
+        <v>1965703.8499999999</v>
+      </c>
+      <c r="D5">
+        <v>2821046.87</v>
+      </c>
+      <c r="E5">
+        <v>3714647.68</v>
+      </c>
+      <c r="F5">
+        <v>4573876.62</v>
+      </c>
+      <c r="G5">
+        <v>5308985.4800000004</v>
+      </c>
+      <c r="H5">
+        <v>5873775.6100000003</v>
+      </c>
+      <c r="I5">
+        <v>6915715.3300000001</v>
+      </c>
+      <c r="J5">
+        <v>7817058.5499999998</v>
+      </c>
+      <c r="K5">
+        <v>8650654.1799999997</v>
+      </c>
+      <c r="L5">
+        <v>9467523.8599999994</v>
+      </c>
+      <c r="M5">
+        <v>10090938.869999999</v>
+      </c>
+      <c r="N5">
+        <v>10090938.869999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>2018</v>
+      </c>
+      <c r="B6">
+        <v>762199.29</v>
+      </c>
+      <c r="C6">
+        <v>1455236.38</v>
+      </c>
+      <c r="D6">
+        <v>2257458.2999999998</v>
+      </c>
+      <c r="E6">
+        <v>2873632.86</v>
+      </c>
+      <c r="F6">
+        <v>3672595.29</v>
+      </c>
+      <c r="G6">
+        <v>4488813</v>
+      </c>
+      <c r="H6">
+        <v>5302322.29</v>
+      </c>
+      <c r="I6">
+        <v>6154741.7199999997</v>
+      </c>
+      <c r="J6">
+        <v>6850908.21</v>
+      </c>
+      <c r="K6">
+        <v>7710664.3399999999</v>
+      </c>
+      <c r="L6">
+        <v>8400932.959999999</v>
+      </c>
+      <c r="M6">
+        <v>9045765.4499999993</v>
+      </c>
+      <c r="N6">
+        <v>9045765.4499999993</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>